<commit_message>
Fix Cl.6.3 Iyc per clause definition: include web portion below neutral axis
Iyc is the moment of inertia of the compression PORTION of the section
(not just feet+lips) about the gravity axis parallel to the web. Under
uplift that is feet + lips + the sub-segments of both webs from y=0 to
the neutral axis. Applied in the JS engine and the Excel workbook; Cb
tooltip added with the 1.75+1.05(M1/M2)+0.3(M1/M2)^2 <= 2.3 formula.
LTB UR drops 69% -> 61% (was conservative).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ln9LHHzMNh3QDoPGqf5Fdh
</commit_message>
<xml_diff>
--- a/IS801_HAT_Calculator.xlsx
+++ b/IS801_HAT_Calculator.xlsx
@@ -2331,7 +2331,7 @@
     <row r="94">
       <c r="A94" s="5" t="inlineStr">
         <is>
-          <t>(b) Sxc = Zbot (comp.)</t>
+          <t>(b) Sxc = Zbot (Ix/dist to comp. fibre)</t>
         </is>
       </c>
       <c r="B94" s="7">
@@ -2352,11 +2352,11 @@
     <row r="95">
       <c r="A95" s="5" t="inlineStr">
         <is>
-          <t>(b) Iyc = Iycf (comp. portion)</t>
+          <t>(b) Iyc = feet+lips + 2×web below NA</t>
         </is>
       </c>
       <c r="B95" s="7">
-        <f>B58</f>
+        <f>B58+2*(($B$11*((B48/B6)*B34)^3/12)*(B28/B34)^2+(((B48/B6)*B34)*$B$11^3/12)*(B6/B34)^2+((B48/B6)*B34)*$B$11*((B29+(B29-B28*(B48/B6)))/2)^2)</f>
         <v/>
       </c>
       <c r="C95" s="5" t="inlineStr">
@@ -2364,7 +2364,11 @@
           <t>mm⁴</t>
         </is>
       </c>
-      <c r="D95" s="2" t="inlineStr"/>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>comp. portion about gravity axis ∥ web</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Align with office sheet: literal Cl.6.4.1 shear, fix interior crippling term, add Cl.6.4.2/6.4.3/5.2.4 checks
- Shear now literal IS 801 MKS: Fv=min(0.4Fy, 1275*sqrt(Fy)/(h/t)) kgf/cm2
  for h/t<=4590/sqrt(Fy), else 5.85e6/(h/t)^2 (was modern AISI form)
- Interior web crippling stress term corrected to k(1.22-0.22k) (was
  wrongly using the end-reaction k(1.33-0.33k))
- New checks: web bending Fbw=36.56e6/(h/t)^2 (Cl.6.4.2), combined
  bending+shear sqrt((f/Fbw)^2+(fv/Fv)^2) (Cl.6.4.3), flat-width maxima
  w/t<=60 and h/t<=150 (Cl.5.2.4)
- Applied in web tool (overview + detailed) and Excel workbook; verified

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ln9LHHzMNh3QDoPGqf5Fdh
</commit_message>
<xml_diff>
--- a/IS801_HAT_Calculator.xlsx
+++ b/IS801_HAT_Calculator.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q144"/>
+  <dimension ref="A1:Q157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2500,11 +2500,11 @@
     <row r="106">
       <c r="A106" s="5" t="inlineStr">
         <is>
-          <t>limit1 = 2.89√(E/Fy)</t>
+          <t>h/t limit = 4590/√Fy (kgf/cm²)</t>
         </is>
       </c>
       <c r="B106" s="7">
-        <f>2.89*SQRT(B13/B12)</f>
+        <f>4590/SQRT(B115)</f>
         <v/>
       </c>
       <c r="C106" s="5" t="inlineStr"/>
@@ -2513,24 +2513,32 @@
     <row r="107">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>limit2 = 5.34√(E/Fy)</t>
+          <t>Fv (kgf/cm²): ≤lim→min(0.4Fy, 1275√Fy/(h/t)); else 5.85e6/(h/t)²</t>
         </is>
       </c>
       <c r="B107" s="7">
-        <f>5.34*SQRT(B13/B12)</f>
-        <v/>
-      </c>
-      <c r="C107" s="5" t="inlineStr"/>
-      <c r="D107" s="2" t="inlineStr"/>
+        <f>IF(B105&lt;=B106,MIN(0.4*B115,1275*SQRT(B115)/B105),5850000/B105^2)</f>
+        <v/>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>kgf/cm²</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>literal Cl.6.4.1</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>Fv: ≤l1→0.4Fy; ≤l2→0.664√(FyE)/(h/t); else 0.905E/(h/t)²</t>
+          <t>Fv (MPa)</t>
         </is>
       </c>
       <c r="B108" s="7">
-        <f>IF(B105&lt;=B106,0.4*B12,IF(B105&lt;=B107,0.664*SQRT(B12*B13)/B105,0.905*B13/B105^2))</f>
+        <f>B107*0.0980665</f>
         <v/>
       </c>
       <c r="C108" s="5" t="inlineStr">
@@ -2648,7 +2656,7 @@
     <row r="117">
       <c r="A117" s="5" t="inlineStr">
         <is>
-          <t>stress term k(1.33−0.33k)</t>
+          <t>stress end k(1.33−0.33k); int k(1.22−0.22k)</t>
         </is>
       </c>
       <c r="B117" s="7">
@@ -2656,7 +2664,20 @@
         <v/>
       </c>
       <c r="C117" s="5" t="inlineStr"/>
-      <c r="D117" s="2" t="inlineStr"/>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>end term</t>
+        </is>
+      </c>
+      <c r="E117" s="7">
+        <f>B116*(1.22-0.22*B116)</f>
+        <v/>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>int term (E117)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="5" t="inlineStr">
@@ -2708,7 +2729,7 @@
         </is>
       </c>
       <c r="B121" s="7">
-        <f>MAX(0,70*B114^2*(305+2.3*(B18/B11)-0.009*(B18/B11)*B105-0.5*B105)*B117*B119)*2*9.80665/1000</f>
+        <f>MAX(0,70*B114^2*(305+2.3*(B18/B11)-0.009*(B18/B11)*B105-0.5*B105)*E117*B119)*2*9.80665/1000</f>
         <v/>
       </c>
       <c r="C121" s="5" t="inlineStr">
@@ -2881,7 +2902,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>12. SUMMARY OF CHECKS</t>
+          <t>12. WEB BENDING Cl.6.4.2 / COMBINED Cl.6.4.3 / FLAT-WIDTH Cl.5.2.4</t>
         </is>
       </c>
       <c r="B134" s="4" t="n"/>
@@ -2890,199 +2911,409 @@
       <c r="E134" s="4" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="10" t="inlineStr">
-        <is>
-          <t>Check</t>
-        </is>
-      </c>
-      <c r="B135" s="10" t="inlineStr">
-        <is>
-          <t>UR</t>
-        </is>
-      </c>
-      <c r="C135" s="10" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="D135" s="10" t="inlineStr">
-        <is>
-          <t>Clause</t>
+      <c r="A135" s="5" t="inlineStr">
+        <is>
+          <t>Fbw = min(36.56e6/(h/t)² kgf/cm², 0.6Fy)</t>
+        </is>
+      </c>
+      <c r="B135" s="7">
+        <f>MIN(36560000/B105^2*0.0980665,0.6*B12)</f>
+        <v/>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>Cl.6.4.2</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>Effective width (max λ/0.673)</t>
-        </is>
-      </c>
-      <c r="B136" s="11">
-        <f>B83</f>
-        <v/>
-      </c>
-      <c r="C136" s="12">
-        <f>IF(B83&gt;=1,"FAIL",IF(B83&gt;=0.9,"MARGINAL","PASS"))</f>
-        <v/>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>Cl.5.2.1.1</t>
-        </is>
-      </c>
+          <t>Fbw(+⅓ if wind)</t>
+        </is>
+      </c>
+      <c r="B136" s="7">
+        <f>B135*IF(B24=1,4/3,1)</f>
+        <v/>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="5" t="inlineStr">
         <is>
-          <t>Edge stiffener Imin/Is</t>
-        </is>
-      </c>
-      <c r="B137" s="11">
-        <f>B89</f>
-        <v/>
-      </c>
-      <c r="C137" s="12">
-        <f>IF(B89&gt;=1,"FAIL",IF(B89&gt;=0.9,"MARGINAL","PASS"))</f>
-        <v/>
-      </c>
-      <c r="D137" s="2" t="inlineStr">
-        <is>
-          <t>Cl.5.2.2.1</t>
-        </is>
-      </c>
+          <t>UR web bending = f_strong/Fbw</t>
+        </is>
+      </c>
+      <c r="B137" s="7">
+        <f>B69/B136</f>
+        <v/>
+      </c>
+      <c r="C137" s="5" t="inlineStr"/>
+      <c r="D137" s="2" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="5" t="inlineStr">
         <is>
-          <t>Bending biaxial (uplift)</t>
-        </is>
-      </c>
-      <c r="B138" s="11">
-        <f>B71</f>
-        <v/>
-      </c>
-      <c r="C138" s="12">
-        <f>IF(B71&gt;=1,"FAIL",IF(B71&gt;=0.9,"MARGINAL","PASS"))</f>
-        <v/>
-      </c>
-      <c r="D138" s="2" t="inlineStr">
-        <is>
-          <t>Cl.6.1.1</t>
-        </is>
-      </c>
+          <t>fv actual = V/(2·H·t)</t>
+        </is>
+      </c>
+      <c r="B138" s="7">
+        <f>B110*1000/(2*B6*B11)</f>
+        <v/>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>MPa</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="5" t="inlineStr">
         <is>
-          <t>Bending gravity</t>
-        </is>
-      </c>
-      <c r="B139" s="11">
-        <f>B73</f>
-        <v/>
-      </c>
-      <c r="C139" s="12">
-        <f>IF(B73&gt;=1,"FAIL",IF(B73&gt;=0.9,"MARGINAL","PASS"))</f>
-        <v/>
-      </c>
+          <t>UR combined = √((f/Fbw)²+(fv/Fv)²)</t>
+        </is>
+      </c>
+      <c r="B139" s="7">
+        <f>SQRT((B69/B136)^2+(B138/(B108*IF(B24=1,4/3,1)))^2)</f>
+        <v/>
+      </c>
+      <c r="C139" s="5" t="inlineStr"/>
       <c r="D139" s="2" t="inlineStr">
         <is>
-          <t>Cl.6.1.1</t>
+          <t>Cl.6.4.3</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="5" t="inlineStr">
         <is>
-          <t>LTB (governing of 2 methods)</t>
-        </is>
-      </c>
-      <c r="B140" s="11">
-        <f>B102</f>
-        <v/>
-      </c>
-      <c r="C140" s="12">
-        <f>IF(B102&gt;=1,"FAIL",IF(B102&gt;=0.9,"MARGINAL","PASS"))</f>
-        <v/>
-      </c>
+          <t>UR flange w/t ≤ 60</t>
+        </is>
+      </c>
+      <c r="B140" s="7">
+        <f>(B8/B11)/60</f>
+        <v/>
+      </c>
+      <c r="C140" s="5" t="inlineStr"/>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Cl.6.3</t>
+          <t>Cl.5.2.4</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="5" t="inlineStr">
         <is>
+          <t>UR web h/t ≤ 150</t>
+        </is>
+      </c>
+      <c r="B141" s="7">
+        <f>B105/150</f>
+        <v/>
+      </c>
+      <c r="C141" s="5" t="inlineStr"/>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>Cl.5.2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="3" t="inlineStr">
+        <is>
+          <t>13. SUMMARY OF CHECKS</t>
+        </is>
+      </c>
+      <c r="B143" s="4" t="n"/>
+      <c r="C143" s="4" t="n"/>
+      <c r="D143" s="4" t="n"/>
+      <c r="E143" s="4" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="10" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B144" s="10" t="inlineStr">
+        <is>
+          <t>UR</t>
+        </is>
+      </c>
+      <c r="C144" s="10" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D144" s="10" t="inlineStr">
+        <is>
+          <t>Clause</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="5" t="inlineStr">
+        <is>
+          <t>Effective width (max λ/0.673)</t>
+        </is>
+      </c>
+      <c r="B145" s="11">
+        <f>B83</f>
+        <v/>
+      </c>
+      <c r="C145" s="12">
+        <f>IF(B83&gt;=1,"FAIL",IF(B83&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>Cl.5.2.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="5" t="inlineStr">
+        <is>
+          <t>Edge stiffener Imin/Is</t>
+        </is>
+      </c>
+      <c r="B146" s="11">
+        <f>B89</f>
+        <v/>
+      </c>
+      <c r="C146" s="12">
+        <f>IF(B89&gt;=1,"FAIL",IF(B89&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>Cl.5.2.2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="5" t="inlineStr">
+        <is>
+          <t>Bending biaxial (uplift)</t>
+        </is>
+      </c>
+      <c r="B147" s="11">
+        <f>B71</f>
+        <v/>
+      </c>
+      <c r="C147" s="12">
+        <f>IF(B71&gt;=1,"FAIL",IF(B71&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>Cl.6.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="5" t="inlineStr">
+        <is>
+          <t>Bending gravity</t>
+        </is>
+      </c>
+      <c r="B148" s="11">
+        <f>B73</f>
+        <v/>
+      </c>
+      <c r="C148" s="12">
+        <f>IF(B73&gt;=1,"FAIL",IF(B73&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>Cl.6.1.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="5" t="inlineStr">
+        <is>
+          <t>LTB (governing of 2 methods)</t>
+        </is>
+      </c>
+      <c r="B149" s="11">
+        <f>B102</f>
+        <v/>
+      </c>
+      <c r="C149" s="12">
+        <f>IF(B102&gt;=1,"FAIL",IF(B102&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>Cl.6.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="5" t="inlineStr">
+        <is>
           <t>Shear</t>
         </is>
       </c>
-      <c r="B141" s="11">
+      <c r="B150" s="11">
         <f>B111</f>
         <v/>
       </c>
-      <c r="C141" s="12">
+      <c r="C150" s="12">
         <f>IF(B111&gt;=1,"FAIL",IF(B111&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
-      <c r="D141" s="2" t="inlineStr">
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>Cl.6.4.1</t>
         </is>
       </c>
     </row>
-    <row r="142">
-      <c r="A142" s="5" t="inlineStr">
+    <row r="151">
+      <c r="A151" s="5" t="inlineStr">
         <is>
           <t>Web crippling (gravity bearing)</t>
         </is>
       </c>
-      <c r="B142" s="11">
+      <c r="B151" s="11">
         <f>B124</f>
         <v/>
       </c>
-      <c r="C142" s="12">
+      <c r="C151" s="12">
         <f>IF(B124&gt;=1,"FAIL",IF(B124&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
-      <c r="D142" s="2" t="inlineStr">
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>Cl.6.5</t>
         </is>
       </c>
     </row>
-    <row r="143">
-      <c r="A143" s="5" t="inlineStr">
+    <row r="152">
+      <c r="A152" s="5" t="inlineStr">
+        <is>
+          <t>Web bending</t>
+        </is>
+      </c>
+      <c r="B152" s="11">
+        <f>B137</f>
+        <v/>
+      </c>
+      <c r="C152" s="12">
+        <f>IF(B137&gt;=1,"FAIL",IF(B137&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>Cl.6.4.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="5" t="inlineStr">
+        <is>
+          <t>Combined bending + shear</t>
+        </is>
+      </c>
+      <c r="B153" s="11">
+        <f>B139</f>
+        <v/>
+      </c>
+      <c r="C153" s="12">
+        <f>IF(B139&gt;=1,"FAIL",IF(B139&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>Cl.6.4.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="5" t="inlineStr">
+        <is>
+          <t>Flange w/t ≤ 60</t>
+        </is>
+      </c>
+      <c r="B154" s="11">
+        <f>B140</f>
+        <v/>
+      </c>
+      <c r="C154" s="12">
+        <f>IF(B140&gt;=1,"FAIL",IF(B140&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>Cl.5.2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="5" t="inlineStr">
+        <is>
+          <t>Web h/t ≤ 150</t>
+        </is>
+      </c>
+      <c r="B155" s="11">
+        <f>B141</f>
+        <v/>
+      </c>
+      <c r="C155" s="12">
+        <f>IF(B141&gt;=1,"FAIL",IF(B141&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>Cl.5.2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="5" t="inlineStr">
         <is>
           <t>Deflection</t>
         </is>
       </c>
-      <c r="B143" s="11">
+      <c r="B156" s="11">
         <f>B132</f>
         <v/>
       </c>
-      <c r="C143" s="12">
+      <c r="C156" s="12">
         <f>IF(B132&gt;=1,"FAIL",IF(B132&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
-      <c r="D143" s="2" t="inlineStr">
+      <c r="D156" s="2" t="inlineStr">
         <is>
           <t>serviceability</t>
         </is>
       </c>
     </row>
-    <row r="144">
-      <c r="A144" s="13" t="inlineStr">
+    <row r="157">
+      <c r="A157" s="13" t="inlineStr">
         <is>
           <t>OVERALL (max UR)</t>
         </is>
       </c>
-      <c r="B144" s="14">
-        <f>MAX(B83,B89,B71,B73,B102,B111,B124,B132)</f>
-        <v/>
-      </c>
-      <c r="C144" s="15">
-        <f>IF(B144&gt;=1,"FAIL",IF(B144&gt;=0.9,"MARGINAL","PASS"))</f>
+      <c r="B157" s="14">
+        <f>MAX(B83,B89,B71,B73,B102,B111,B124,B137,B139,B140,B141,B132)</f>
+        <v/>
+      </c>
+      <c r="C157" s="15">
+        <f>IF(B157&gt;=1,"FAIL",IF(B157&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove 33% wind increase from all allowables (project practice)
All checks now use plain 0.6Fy-based allowables in both the web tool and
the Excel workbook. windPlus paths retained but permanently off.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ln9LHHzMNh3QDoPGqf5Fdh
</commit_message>
<xml_diff>
--- a/IS801_HAT_Calculator.xlsx
+++ b/IS801_HAT_Calculator.xlsx
@@ -849,16 +849,16 @@
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Wind/seismic combo? (1=yes → +⅓ allowable)</t>
+          <t>Wind +33% allowable increase</t>
         </is>
       </c>
       <c r="B24" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C24" s="5" t="inlineStr"/>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>IS 800/875 WSM practice</t>
+          <t>REMOVED per project practice — allowables at 0.6Fy</t>
         </is>
       </c>
     </row>
@@ -1940,11 +1940,11 @@
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fb(+⅓ if wind) </t>
+          <t>Fb design (no wind increase)</t>
         </is>
       </c>
       <c r="B66" s="7">
-        <f>B65*IF(B24=1,4/3,1)</f>
+        <f>B65</f>
         <v/>
       </c>
       <c r="C66" s="5" t="inlineStr">
@@ -1952,11 +1952,7 @@
           <t>MPa</t>
         </is>
       </c>
-      <c r="D66" s="2" t="inlineStr">
-        <is>
-          <t>IS 800/875 WSM</t>
-        </is>
-      </c>
+      <c r="D66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
@@ -2029,7 +2025,7 @@
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>UR bending (biaxial) = (f_strong+f_weak)/Fb(+⅓)</t>
+          <t>UR bending (biaxial) = (f_strong+f_weak)/Fb</t>
         </is>
       </c>
       <c r="B71" s="7">
@@ -2446,11 +2442,11 @@
     <row r="101">
       <c r="A101" s="5" t="inlineStr">
         <is>
-          <t>Fb_LTB(+⅓ if wind)</t>
+          <t>Fb_LTB design (no wind increase)</t>
         </is>
       </c>
       <c r="B101" s="7">
-        <f>B100*IF(B24=1,4/3,1)</f>
+        <f>B100</f>
         <v/>
       </c>
       <c r="C101" s="5" t="inlineStr">
@@ -2463,7 +2459,7 @@
     <row r="102">
       <c r="A102" s="5" t="inlineStr">
         <is>
-          <t>UR LTB = f_bot/Fb_LTB(+⅓)</t>
+          <t>UR LTB = f_bot/Fb_LTB</t>
         </is>
       </c>
       <c r="B102" s="7">
@@ -2934,11 +2930,11 @@
     <row r="136">
       <c r="A136" s="5" t="inlineStr">
         <is>
-          <t>Fbw(+⅓ if wind)</t>
+          <t>Fbw design (no wind increase)</t>
         </is>
       </c>
       <c r="B136" s="7">
-        <f>B135*IF(B24=1,4/3,1)</f>
+        <f>B135</f>
         <v/>
       </c>
       <c r="C136" s="5" t="inlineStr">
@@ -2985,7 +2981,7 @@
         </is>
       </c>
       <c r="B139" s="7">
-        <f>SQRT((B69/B136)^2+(B138/(B108*IF(B24=1,4/3,1)))^2)</f>
+        <f>SQRT((B69/B136)^2+(B138/B108)^2)</f>
         <v/>
       </c>
       <c r="C139" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Separate web-crippling checks: overhang (cantilever end) vs inner span
Adds an Overhang Lo input. The overhang/end support gets the cantilever
web-crippling formula (98+4.2N/t..., k(1.33-0.33k), 1.15-0.15r/t) with
reaction w(Lo+L)^2/(2L); inner spans get the interior formula (305+2.3N/t...,
k(1.22-0.22k), 1.06-0.06r/t) with the continuous-support reaction. Inner
check shows N/A for a simply-supported single span. Applied in the web
tool (overview + detailed, two panels) and the Excel workbook.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ln9LHHzMNh3QDoPGqf5Fdh
</commit_message>
<xml_diff>
--- a/IS801_HAT_Calculator.xlsx
+++ b/IS801_HAT_Calculator.xlsx
@@ -493,7 +493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q157"/>
+  <dimension ref="A1:Q158"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -862,6 +862,26 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Overhang Lo (m)</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>cantilever past end rafter; 0=none</t>
+        </is>
+      </c>
+    </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
@@ -2738,11 +2758,11 @@
     <row r="122">
       <c r="A122" s="5" t="inlineStr">
         <is>
-          <t>R_end (gravity) coeff·w·L</t>
+          <t>R_overhang (gravity)</t>
         </is>
       </c>
       <c r="B122" s="7">
-        <f>IF(B15="2-span continuous",0.375,IF(B15="3+ span continuous",0.4,0.5))*B22*B14</f>
+        <f>IF(B25&gt;0,B22*(B25+B14)^2/(2*B14),IF(B15="2-span continuous",0.375,IF(B15="3+ span continuous",0.4,0.5))*B22*B14)</f>
         <v/>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -2750,12 +2770,16 @@
           <t>kN</t>
         </is>
       </c>
-      <c r="D122" s="2" t="inlineStr"/>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>Lo&gt;0: w(Lo+L)²/2L (cantilever end)</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="5" t="inlineStr">
         <is>
-          <t>R_int (gravity)</t>
+          <t>R_inner span (gravity)</t>
         </is>
       </c>
       <c r="B123" s="7">
@@ -2772,17 +2796,34 @@
     <row r="124">
       <c r="A124" s="5" t="inlineStr">
         <is>
-          <t>UR web crippling = max(Rend/Pend, Rint/Pint)</t>
+          <t>UR web crippling — OVERHANG = R_overhang/P_cant</t>
         </is>
       </c>
       <c r="B124" s="7">
-        <f>MAX(B122/B120,IF(B123&gt;0,B123/B121,0))</f>
+        <f>B122/B120</f>
         <v/>
       </c>
       <c r="C124" s="5" t="inlineStr"/>
       <c r="D124" s="2" t="inlineStr">
         <is>
-          <t>uplift reaction → bolt check, not web</t>
+          <t>cantilever end (Cl.6.5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="5" t="inlineStr">
+        <is>
+          <t>UR web crippling — INNER span = R_inner/P_int</t>
+        </is>
+      </c>
+      <c r="B125" s="7">
+        <f>IF(B123&gt;0,B123/B121,0)</f>
+        <v/>
+      </c>
+      <c r="C125" s="5" t="inlineStr"/>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>inner support (Cl.6.5)</t>
         </is>
       </c>
     </row>
@@ -3181,7 +3222,7 @@
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
         <is>
-          <t>Web crippling (gravity bearing)</t>
+          <t>Web crippling — overhang (cantilever end)</t>
         </is>
       </c>
       <c r="B151" s="11">
@@ -3201,75 +3242,75 @@
     <row r="152">
       <c r="A152" s="5" t="inlineStr">
         <is>
-          <t>Web bending</t>
+          <t>Web crippling — inner span</t>
         </is>
       </c>
       <c r="B152" s="11">
-        <f>B137</f>
+        <f>B125</f>
         <v/>
       </c>
       <c r="C152" s="12">
-        <f>IF(B137&gt;=1,"FAIL",IF(B137&gt;=0.9,"MARGINAL","PASS"))</f>
+        <f>IF(B125&gt;=1,"FAIL",IF(B125&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
       <c r="D152" s="2" t="inlineStr">
         <is>
-          <t>Cl.6.4.2</t>
+          <t>Cl.6.5</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="5" t="inlineStr">
         <is>
-          <t>Combined bending + shear</t>
+          <t>Web bending</t>
         </is>
       </c>
       <c r="B153" s="11">
-        <f>B139</f>
+        <f>B137</f>
         <v/>
       </c>
       <c r="C153" s="12">
-        <f>IF(B139&gt;=1,"FAIL",IF(B139&gt;=0.9,"MARGINAL","PASS"))</f>
+        <f>IF(B137&gt;=1,"FAIL",IF(B137&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
       <c r="D153" s="2" t="inlineStr">
         <is>
-          <t>Cl.6.4.3</t>
+          <t>Cl.6.4.2</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="5" t="inlineStr">
         <is>
-          <t>Flange w/t ≤ 60</t>
+          <t>Combined bending + shear</t>
         </is>
       </c>
       <c r="B154" s="11">
-        <f>B140</f>
+        <f>B139</f>
         <v/>
       </c>
       <c r="C154" s="12">
-        <f>IF(B140&gt;=1,"FAIL",IF(B140&gt;=0.9,"MARGINAL","PASS"))</f>
+        <f>IF(B139&gt;=1,"FAIL",IF(B139&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
       <c r="D154" s="2" t="inlineStr">
         <is>
-          <t>Cl.5.2.4</t>
+          <t>Cl.6.4.3</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="5" t="inlineStr">
         <is>
-          <t>Web h/t ≤ 150</t>
+          <t>Flange w/t ≤ 60</t>
         </is>
       </c>
       <c r="B155" s="11">
-        <f>B141</f>
+        <f>B140</f>
         <v/>
       </c>
       <c r="C155" s="12">
-        <f>IF(B141&gt;=1,"FAIL",IF(B141&gt;=0.9,"MARGINAL","PASS"))</f>
+        <f>IF(B140&gt;=1,"FAIL",IF(B140&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -3281,35 +3322,55 @@
     <row r="156">
       <c r="A156" s="5" t="inlineStr">
         <is>
+          <t>Web h/t ≤ 150</t>
+        </is>
+      </c>
+      <c r="B156" s="11">
+        <f>B141</f>
+        <v/>
+      </c>
+      <c r="C156" s="12">
+        <f>IF(B141&gt;=1,"FAIL",IF(B141&gt;=0.9,"MARGINAL","PASS"))</f>
+        <v/>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>Cl.5.2.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="5" t="inlineStr">
+        <is>
           <t>Deflection</t>
         </is>
       </c>
-      <c r="B156" s="11">
+      <c r="B157" s="11">
         <f>B132</f>
         <v/>
       </c>
-      <c r="C156" s="12">
+      <c r="C157" s="12">
         <f>IF(B132&gt;=1,"FAIL",IF(B132&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
-      <c r="D156" s="2" t="inlineStr">
+      <c r="D157" s="2" t="inlineStr">
         <is>
           <t>serviceability</t>
         </is>
       </c>
     </row>
-    <row r="157">
-      <c r="A157" s="13" t="inlineStr">
+    <row r="158">
+      <c r="A158" s="13" t="inlineStr">
         <is>
           <t>OVERALL (max UR)</t>
         </is>
       </c>
-      <c r="B157" s="14">
-        <f>MAX(B83,B89,B71,B73,B102,B111,B124,B137,B139,B140,B141,B132)</f>
-        <v/>
-      </c>
-      <c r="C157" s="15">
-        <f>IF(B157&gt;=1,"FAIL",IF(B157&gt;=0.9,"MARGINAL","PASS"))</f>
+      <c r="B158" s="14">
+        <f>MAX(B83,B89,B71,B73,B102,B111,B124,B125,B137,B139,B140,B141,B132)</f>
+        <v/>
+      </c>
+      <c r="C158" s="15">
+        <f>IF(B158&gt;=1,"FAIL",IF(B158&gt;=0.9,"MARGINAL","PASS"))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Explicit load combinations: Uplift = WL up - DL, Downward = WL down + DL
UDL panel now takes DL, wind uplift, and wind downward separately and
derives the two design combinations live (deriveCombos): net uplift
(hogging) and downward (sagging). Both drive their respective checks;
bending rows relabelled Uplift combo / Downward combo. Applied in the
web tool and the Excel workbook (DL at B21, WL up B22, WL down G22).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ln9LHHzMNh3QDoPGqf5Fdh
</commit_message>
<xml_diff>
--- a/IS801_HAT_Calculator.xlsx
+++ b/IS801_HAT_Calculator.xlsx
@@ -797,11 +797,11 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>w net uplift (working)</t>
+          <t>Dead load DL</t>
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.981</v>
+        <v>0.147</v>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
@@ -810,25 +810,37 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>WL−DL, service</t>
+          <t>resists uplift, adds to downward</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>w gravity (working)</t>
+          <t>Wind uplift WL↑ (gross)</t>
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>0.147</v>
+        <v>1.128</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
           <t>kN/m</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>suction, upward</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Wind down WL↓</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1888,7 +1900,7 @@
         </is>
       </c>
       <c r="B62" s="7">
-        <f>B21*B14^2/8</f>
+        <f>MAX(B22-B21,0)*B14^2/8</f>
         <v/>
       </c>
       <c r="C62" s="5" t="inlineStr">
@@ -1898,18 +1910,18 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>wL²/8: exact 2-span support M, conservative 3+</t>
+          <t>UPLIFT combo (WL↑−DL); wL²/8</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>M gravity = w·L²/8</t>
+          <t>M downward = (WL↓+DL)·L²/8</t>
         </is>
       </c>
       <c r="B63" s="7">
-        <f>B22*B14^2/8</f>
+        <f>(G22+B21)*B14^2/8</f>
         <v/>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -1917,7 +1929,11 @@
           <t>kN·m</t>
         </is>
       </c>
-      <c r="D63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>DOWNWARD combo</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
@@ -2762,7 +2778,7 @@
         </is>
       </c>
       <c r="B122" s="7">
-        <f>IF(B25&gt;0,B22*(B25+B14)^2/(2*B14),IF(B15="2-span continuous",0.375,IF(B15="3+ span continuous",0.4,0.5))*B22*B14)</f>
+        <f>IF(B25&gt;0,(G22+B21)*(B25+B14)^2/(2*B14),IF(B15="2-span continuous",0.375,IF(B15="3+ span continuous",0.4,0.5))*(G22+B21)*B14)</f>
         <v/>
       </c>
       <c r="C122" s="5" t="inlineStr">
@@ -2783,7 +2799,7 @@
         </is>
       </c>
       <c r="B123" s="7">
-        <f>IF(B15="2-span continuous",1.25,IF(B15="3+ span continuous",1.1,0))*B22*B14</f>
+        <f>IF(B15="2-span continuous",1.25,IF(B15="3+ span continuous",1.1,0))*(G22+B21)*B14</f>
         <v/>
       </c>
       <c r="C123" s="5" t="inlineStr">
@@ -2858,7 +2874,7 @@
         </is>
       </c>
       <c r="B128" s="7">
-        <f>B127*ABS(B21)*(B14*1000)^4/(B13*B49)</f>
+        <f>B127*MAX(B22-B21,0)*(B14*1000)^4/(B13*B49)</f>
         <v/>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -2868,7 +2884,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>1 kN/m = 1 N/mm</t>
+          <t>uplift combo; 1 kN/m=1 N/mm</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reconcile Configuration-panel deflection with Serviceability check
Both now use the governing combo load (max of uplift/downward), not uplift
alone. Configuration panel: Simple Span = simply-supported idealisation
(5/384) with allowable row added; note explains it equals the Serviceability
value when support=simply supported, and why continuity makes them differ.
Serviceability row relabelled 'as-configured' and states the governing
combo load. Excel deflection uses governing combo too.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ln9LHHzMNh3QDoPGqf5Fdh
</commit_message>
<xml_diff>
--- a/IS801_HAT_Calculator.xlsx
+++ b/IS801_HAT_Calculator.xlsx
@@ -2874,7 +2874,7 @@
         </is>
       </c>
       <c r="B128" s="7">
-        <f>B127*MAX(B22-B21,0)*(B14*1000)^4/(B13*B49)</f>
+        <f>B127*MAX(MAX(B22-B21,0),G22+B21)*(B14*1000)^4/(B13*B49)</f>
         <v/>
       </c>
       <c r="C128" s="5" t="inlineStr">
@@ -2884,7 +2884,7 @@
       </c>
       <c r="D128" s="2" t="inlineStr">
         <is>
-          <t>uplift combo; 1 kN/m=1 N/mm</t>
+          <t>governing combo; 1 kN/m=1 N/mm</t>
         </is>
       </c>
     </row>

</xml_diff>